<commit_message>
fix errors qa fdb3f2aabdff688dee53454544999ef87c067347
</commit_message>
<xml_diff>
--- a/qaFHIRErrors/ig/StructureDefinition-fr-service-request-document.xlsx
+++ b/qaFHIRErrors/ig/StructureDefinition-fr-service-request-document.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AO$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AO$66</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2422" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2460" uniqueCount="506">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-26T13:43:53+00:00</t>
+    <t>2026-08-26T14:38:07+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -659,6 +659,28 @@
   <si>
     <t>base64Binary
 booleancanonicalcodedatedateTimedecimalidinstantintegermarkdownoidpositiveIntstringtimeunsignedInturiurluuidAddressAgeAnnotationAttachmentCodeableConceptCodingContactPointCountDistanceDurationHumanNameIdentifierMoneyPeriodQuantityRangeRatioReferenceSampledDataSignatureTimingContactDetailContributorDataRequirementExpressionParameterDefinitionRelatedArtifactTriggerDefinitionUsageContextDosageMeta</t>
+  </si>
+  <si>
+    <t>ServiceRequest.extension:reason</t>
+  </si>
+  <si>
+    <t>reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {http://hl7.org/fhir/5.0/StructureDefinition/extension-ServiceRequest.reason|0.1.0}
+</t>
+  </si>
+  <si>
+    <t>R5: Explanation/Justification for procedure or service additional types</t>
+  </si>
+  <si>
+    <t>R5: `ServiceRequest.reason` additional types (CodeableReference(http://hl7.org/fhir/StructureDefinition/Condition), CodeableReference(http://hl7.org/fhir/StructureDefinition/Observation), CodeableReference(http://hl7.org/fhir/StructureDefinition/DiagnosticReport), CodeableReference(http://hl7.org/fhir/StructureDefinition/DocumentReference), CodeableReference(http://hl7.org/fhir/StructureDefinition/DetectedIssue))</t>
+  </si>
+  <si>
+    <t>Element `ServiceRequest.reason` is mapped to FHIR R4 element `ServiceRequest.reasonCode` as `SourceIsBroaderThanTarget`.
+Element `ServiceRequest.reason` is mapped to FHIR R4 element `ServiceRequest.reasonReference` as `SourceIsBroaderThanTarget`.
+The mappings for `ServiceRequest.reason` do not cover the following types: CodeableReference.
+This element represents why the referral is being made and may be used to decide how the service will be performed, or even if it will be performed at all. To be as specific as possible,  a reference to  *Observation* or *Condition* should be used if available.  Otherwise, use `concept.text` element if the data is free (uncoded) text as shown in the [CT Scan example](https://hl7.org/fhir/servicerequest-example-di.html).</t>
   </si>
   <si>
     <t>ServiceRequest.modifierExtension</t>
@@ -1894,7 +1916,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AO65"/>
+  <dimension ref="A1:AO66"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="51.5" customWidth="true" bestFit="true"/>
@@ -5428,11 +5450,13 @@
         <v>207</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>207</v>
-      </c>
-      <c r="C31" s="2"/>
+        <v>134</v>
+      </c>
+      <c r="C31" t="s" s="2">
+        <v>208</v>
+      </c>
       <c r="D31" t="s" s="2">
-        <v>208</v>
+        <v>81</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
@@ -5445,26 +5469,24 @@
         <v>81</v>
       </c>
       <c r="I31" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="J31" t="s" s="2">
         <v>81</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>135</v>
+        <v>209</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="N31" t="s" s="2">
-        <v>211</v>
-      </c>
-      <c r="O31" t="s" s="2">
         <v>212</v>
       </c>
+      <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
         <v>81</v>
       </c>
@@ -5512,7 +5534,7 @@
         <v>81</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>213</v>
+        <v>140</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>79</v>
@@ -5521,7 +5543,7 @@
         <v>80</v>
       </c>
       <c r="AI31" t="s" s="2">
-        <v>81</v>
+        <v>147</v>
       </c>
       <c r="AJ31" t="s" s="2">
         <v>141</v>
@@ -5533,7 +5555,7 @@
         <v>81</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>133</v>
+        <v>81</v>
       </c>
       <c r="AN31" t="s" s="2">
         <v>81</v>
@@ -5544,14 +5566,14 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>81</v>
+        <v>214</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
@@ -5564,24 +5586,26 @@
         <v>81</v>
       </c>
       <c r="I32" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="K32" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L32" t="s" s="2">
         <v>215</v>
       </c>
-      <c r="L32" t="s" s="2">
+      <c r="M32" t="s" s="2">
         <v>216</v>
       </c>
-      <c r="M32" t="s" s="2">
+      <c r="N32" t="s" s="2">
         <v>217</v>
       </c>
-      <c r="N32" t="s" s="2">
+      <c r="O32" t="s" s="2">
         <v>218</v>
       </c>
-      <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
         <v>81</v>
       </c>
@@ -5617,17 +5641,19 @@
         <v>81</v>
       </c>
       <c r="AB32" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC32" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD32" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE32" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF32" t="s" s="2">
         <v>219</v>
-      </c>
-      <c r="AC32" s="2"/>
-      <c r="AD32" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE32" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="AF32" t="s" s="2">
-        <v>214</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>79</v>
@@ -5639,34 +5665,32 @@
         <v>81</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>102</v>
+        <v>141</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>220</v>
+        <v>81</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>221</v>
+        <v>81</v>
       </c>
       <c r="AM32" t="s" s="2">
-        <v>222</v>
+        <v>133</v>
       </c>
       <c r="AN32" t="s" s="2">
-        <v>223</v>
+        <v>81</v>
       </c>
       <c r="AO32" t="s" s="2">
-        <v>224</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>214</v>
-      </c>
-      <c r="C33" t="s" s="2">
-        <v>226</v>
-      </c>
+        <v>220</v>
+      </c>
+      <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
         <v>81</v>
       </c>
@@ -5675,7 +5699,7 @@
         <v>79</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>81</v>
@@ -5687,16 +5711,16 @@
         <v>91</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -5734,19 +5758,17 @@
         <v>81</v>
       </c>
       <c r="AB33" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC33" t="s" s="2">
-        <v>81</v>
-      </c>
+        <v>225</v>
+      </c>
+      <c r="AC33" s="2"/>
       <c r="AD33" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE33" t="s" s="2">
-        <v>81</v>
+        <v>139</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>79</v>
@@ -5761,29 +5783,31 @@
         <v>102</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="AN33" t="s" s="2">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="AO33" t="s" s="2">
-        <v>224</v>
+        <v>230</v>
       </c>
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>229</v>
-      </c>
-      <c r="C34" s="2"/>
+        <v>220</v>
+      </c>
+      <c r="C34" t="s" s="2">
+        <v>232</v>
+      </c>
       <c r="D34" t="s" s="2">
         <v>81</v>
       </c>
@@ -5792,7 +5816,7 @@
         <v>79</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>81</v>
@@ -5804,16 +5828,16 @@
         <v>91</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
@@ -5863,7 +5887,7 @@
         <v>81</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>79</v>
@@ -5878,27 +5902,27 @@
         <v>102</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>81</v>
+        <v>229</v>
       </c>
       <c r="AO34" t="s" s="2">
-        <v>81</v>
+        <v>230</v>
       </c>
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5921,16 +5945,16 @@
         <v>91</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>104</v>
+        <v>236</v>
       </c>
       <c r="L35" t="s" s="2">
+        <v>237</v>
+      </c>
+      <c r="M35" t="s" s="2">
         <v>238</v>
       </c>
-      <c r="M35" t="s" s="2">
+      <c r="N35" t="s" s="2">
         <v>239</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>240</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5980,7 +6004,7 @@
         <v>81</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>79</v>
@@ -5995,13 +6019,13 @@
         <v>102</v>
       </c>
       <c r="AK35" t="s" s="2">
+        <v>240</v>
+      </c>
+      <c r="AL35" t="s" s="2">
         <v>241</v>
       </c>
-      <c r="AL35" t="s" s="2">
-        <v>235</v>
-      </c>
       <c r="AM35" t="s" s="2">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="AN35" t="s" s="2">
         <v>81</v>
@@ -6012,14 +6036,14 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
-        <v>243</v>
+        <v>81</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
@@ -6038,15 +6062,17 @@
         <v>91</v>
       </c>
       <c r="K36" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="L36" t="s" s="2">
         <v>244</v>
       </c>
-      <c r="L36" t="s" s="2">
+      <c r="M36" t="s" s="2">
         <v>245</v>
       </c>
-      <c r="M36" t="s" s="2">
+      <c r="N36" t="s" s="2">
         <v>246</v>
       </c>
-      <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>81</v>
@@ -6095,7 +6121,7 @@
         <v>81</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>79</v>
@@ -6113,10 +6139,10 @@
         <v>247</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="AN36" t="s" s="2">
         <v>81</v>
@@ -6127,14 +6153,14 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
@@ -6153,13 +6179,13 @@
         <v>91</v>
       </c>
       <c r="K37" t="s" s="2">
+        <v>250</v>
+      </c>
+      <c r="L37" t="s" s="2">
+        <v>251</v>
+      </c>
+      <c r="M37" t="s" s="2">
         <v>252</v>
-      </c>
-      <c r="L37" t="s" s="2">
-        <v>253</v>
-      </c>
-      <c r="M37" t="s" s="2">
-        <v>254</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -6210,7 +6236,7 @@
         <v>81</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>79</v>
@@ -6225,13 +6251,13 @@
         <v>102</v>
       </c>
       <c r="AK37" t="s" s="2">
+        <v>253</v>
+      </c>
+      <c r="AL37" t="s" s="2">
+        <v>254</v>
+      </c>
+      <c r="AM37" t="s" s="2">
         <v>255</v>
-      </c>
-      <c r="AL37" t="s" s="2">
-        <v>256</v>
-      </c>
-      <c r="AM37" t="s" s="2">
-        <v>257</v>
       </c>
       <c r="AN37" t="s" s="2">
         <v>81</v>
@@ -6242,21 +6268,21 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H38" t="s" s="2">
         <v>81</v>
@@ -6268,20 +6294,16 @@
         <v>91</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>215</v>
+        <v>258</v>
       </c>
       <c r="L38" t="s" s="2">
+        <v>259</v>
+      </c>
+      <c r="M38" t="s" s="2">
         <v>260</v>
       </c>
-      <c r="M38" t="s" s="2">
-        <v>261</v>
-      </c>
-      <c r="N38" t="s" s="2">
-        <v>262</v>
-      </c>
-      <c r="O38" t="s" s="2">
-        <v>263</v>
-      </c>
+      <c r="N38" s="2"/>
+      <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
         <v>81</v>
       </c>
@@ -6329,13 +6351,13 @@
         <v>81</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AI38" t="s" s="2">
         <v>81</v>
@@ -6344,13 +6366,13 @@
         <v>102</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="AN38" t="s" s="2">
         <v>81</v>
@@ -6361,18 +6383,18 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
-        <v>81</v>
+        <v>265</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="G39" t="s" s="2">
         <v>90</v>
@@ -6381,24 +6403,26 @@
         <v>81</v>
       </c>
       <c r="I39" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="J39" t="s" s="2">
         <v>91</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>110</v>
+        <v>221</v>
       </c>
       <c r="L39" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="M39" t="s" s="2">
+        <v>267</v>
+      </c>
+      <c r="N39" t="s" s="2">
         <v>268</v>
       </c>
-      <c r="M39" t="s" s="2">
+      <c r="O39" t="s" s="2">
         <v>269</v>
       </c>
-      <c r="N39" t="s" s="2">
-        <v>270</v>
-      </c>
-      <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>81</v>
       </c>
@@ -6422,13 +6446,13 @@
         <v>81</v>
       </c>
       <c r="X39" t="s" s="2">
-        <v>182</v>
+        <v>81</v>
       </c>
       <c r="Y39" t="s" s="2">
-        <v>271</v>
+        <v>81</v>
       </c>
       <c r="Z39" t="s" s="2">
-        <v>272</v>
+        <v>81</v>
       </c>
       <c r="AA39" t="s" s="2">
         <v>81</v>
@@ -6446,10 +6470,10 @@
         <v>81</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AG39" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="AH39" t="s" s="2">
         <v>90</v>
@@ -6461,27 +6485,27 @@
         <v>102</v>
       </c>
       <c r="AK39" t="s" s="2">
+        <v>270</v>
+      </c>
+      <c r="AL39" t="s" s="2">
+        <v>271</v>
+      </c>
+      <c r="AM39" t="s" s="2">
+        <v>272</v>
+      </c>
+      <c r="AN39" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO39" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="40" hidden="true">
+      <c r="A40" t="s" s="2">
         <v>273</v>
       </c>
-      <c r="AL39" t="s" s="2">
-        <v>274</v>
-      </c>
-      <c r="AM39" t="s" s="2">
-        <v>275</v>
-      </c>
-      <c r="AN39" t="s" s="2">
-        <v>276</v>
-      </c>
-      <c r="AO39" t="s" s="2">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="s" s="2">
-        <v>278</v>
-      </c>
       <c r="B40" t="s" s="2">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6495,7 +6519,7 @@
         <v>90</v>
       </c>
       <c r="H40" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="I40" t="s" s="2">
         <v>91</v>
@@ -6507,13 +6531,13 @@
         <v>110</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N40" t="s" s="2">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
@@ -6542,10 +6566,10 @@
         <v>182</v>
       </c>
       <c r="Y40" t="s" s="2">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="Z40" t="s" s="2">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="AA40" t="s" s="2">
         <v>81</v>
@@ -6563,7 +6587,7 @@
         <v>81</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>90</v>
@@ -6578,27 +6602,27 @@
         <v>102</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="AL40" t="s" s="2">
-        <v>133</v>
+        <v>280</v>
       </c>
       <c r="AM40" t="s" s="2">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="AO40" t="s" s="2">
-        <v>81</v>
+        <v>283</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6606,35 +6630,33 @@
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H41" t="s" s="2">
         <v>91</v>
       </c>
       <c r="I41" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="J41" t="s" s="2">
         <v>91</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>192</v>
+        <v>110</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="N41" t="s" s="2">
-        <v>290</v>
-      </c>
-      <c r="O41" t="s" s="2">
-        <v>291</v>
-      </c>
+        <v>287</v>
+      </c>
+      <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>81</v>
       </c>
@@ -6658,13 +6680,13 @@
         <v>81</v>
       </c>
       <c r="X41" t="s" s="2">
-        <v>292</v>
+        <v>182</v>
       </c>
       <c r="Y41" t="s" s="2">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="Z41" t="s" s="2">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="AA41" t="s" s="2">
         <v>81</v>
@@ -6682,13 +6704,13 @@
         <v>81</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="AG41" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="AH41" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AI41" t="s" s="2">
         <v>81</v>
@@ -6697,27 +6719,27 @@
         <v>102</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>81</v>
+        <v>290</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>295</v>
+        <v>133</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="AN41" t="s" s="2">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="AO41" t="s" s="2">
         <v>81</v>
       </c>
     </row>
-    <row r="42" hidden="true">
+    <row r="42">
       <c r="A42" t="s" s="2">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6728,10 +6750,10 @@
         <v>79</v>
       </c>
       <c r="G42" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H42" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="I42" t="s" s="2">
         <v>81</v>
@@ -6740,49 +6762,51 @@
         <v>91</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>110</v>
+        <v>192</v>
       </c>
       <c r="L42" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="M42" t="s" s="2">
+        <v>295</v>
+      </c>
+      <c r="N42" t="s" s="2">
+        <v>296</v>
+      </c>
+      <c r="O42" t="s" s="2">
+        <v>297</v>
+      </c>
+      <c r="P42" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q42" s="2"/>
+      <c r="R42" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S42" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T42" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U42" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V42" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W42" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X42" t="s" s="2">
         <v>298</v>
       </c>
-      <c r="M42" t="s" s="2">
+      <c r="Y42" t="s" s="2">
         <v>299</v>
       </c>
-      <c r="N42" s="2"/>
-      <c r="O42" s="2"/>
-      <c r="P42" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Q42" t="s" s="2">
+      <c r="Z42" t="s" s="2">
         <v>300</v>
       </c>
-      <c r="R42" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="S42" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="T42" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="U42" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="V42" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="W42" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="X42" t="s" s="2">
-        <v>182</v>
-      </c>
-      <c r="Y42" t="s" s="2">
-        <v>301</v>
-      </c>
-      <c r="Z42" t="s" s="2">
-        <v>302</v>
-      </c>
       <c r="AA42" t="s" s="2">
         <v>81</v>
       </c>
@@ -6799,13 +6823,13 @@
         <v>81</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH42" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AI42" t="s" s="2">
         <v>81</v>
@@ -6814,16 +6838,16 @@
         <v>102</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>303</v>
+        <v>81</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>306</v>
+        <v>292</v>
       </c>
       <c r="AO42" t="s" s="2">
         <v>81</v>
@@ -6831,10 +6855,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6851,59 +6875,55 @@
         <v>81</v>
       </c>
       <c r="I43" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="J43" t="s" s="2">
         <v>91</v>
       </c>
       <c r="K43" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="L43" t="s" s="2">
+        <v>304</v>
+      </c>
+      <c r="M43" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="N43" s="2"/>
+      <c r="O43" s="2"/>
+      <c r="P43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q43" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="R43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X43" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="Y43" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="Z43" t="s" s="2">
         <v>308</v>
       </c>
-      <c r="L43" t="s" s="2">
-        <v>309</v>
-      </c>
-      <c r="M43" t="s" s="2">
-        <v>310</v>
-      </c>
-      <c r="N43" t="s" s="2">
-        <v>311</v>
-      </c>
-      <c r="O43" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="P43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Q43" t="s" s="2">
-        <v>313</v>
-      </c>
-      <c r="R43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="S43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="T43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="U43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="V43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="W43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="X43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Y43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Z43" t="s" s="2">
-        <v>81</v>
-      </c>
       <c r="AA43" t="s" s="2">
         <v>81</v>
       </c>
@@ -6920,7 +6940,7 @@
         <v>81</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>79</v>
@@ -6935,65 +6955,69 @@
         <v>102</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>81</v>
+        <v>310</v>
       </c>
       <c r="AM43" t="s" s="2">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="AN43" t="s" s="2">
-        <v>81</v>
+        <v>312</v>
       </c>
       <c r="AO43" t="s" s="2">
         <v>81</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>317</v>
+        <v>81</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="G44" t="s" s="2">
         <v>90</v>
       </c>
       <c r="H44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I44" t="s" s="2">
         <v>91</v>
-      </c>
-      <c r="I44" t="s" s="2">
-        <v>81</v>
       </c>
       <c r="J44" t="s" s="2">
         <v>91</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>192</v>
+        <v>314</v>
       </c>
       <c r="L44" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="M44" t="s" s="2">
+        <v>316</v>
+      </c>
+      <c r="N44" t="s" s="2">
+        <v>317</v>
+      </c>
+      <c r="O44" t="s" s="2">
         <v>318</v>
       </c>
-      <c r="M44" t="s" s="2">
+      <c r="P44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q44" t="s" s="2">
         <v>319</v>
       </c>
-      <c r="N44" t="s" s="2">
-        <v>320</v>
-      </c>
-      <c r="O44" s="2"/>
-      <c r="P44" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Q44" s="2"/>
       <c r="R44" t="s" s="2">
         <v>81</v>
       </c>
@@ -7013,13 +7037,13 @@
         <v>81</v>
       </c>
       <c r="X44" t="s" s="2">
-        <v>292</v>
+        <v>81</v>
       </c>
       <c r="Y44" t="s" s="2">
-        <v>321</v>
+        <v>81</v>
       </c>
       <c r="Z44" t="s" s="2">
-        <v>322</v>
+        <v>81</v>
       </c>
       <c r="AA44" t="s" s="2">
         <v>81</v>
@@ -7037,7 +7061,7 @@
         <v>81</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>79</v>
@@ -7052,38 +7076,38 @@
         <v>102</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="AL44" t="s" s="2">
-        <v>324</v>
+        <v>81</v>
       </c>
       <c r="AM44" t="s" s="2">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="AN44" t="s" s="2">
-        <v>326</v>
+        <v>81</v>
       </c>
       <c r="AO44" t="s" s="2">
-        <v>327</v>
+        <v>81</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H45" t="s" s="2">
         <v>91</v>
@@ -7098,13 +7122,13 @@
         <v>192</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="N45" t="s" s="2">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
@@ -7130,13 +7154,13 @@
         <v>81</v>
       </c>
       <c r="X45" t="s" s="2">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="Y45" t="s" s="2">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="Z45" t="s" s="2">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="AA45" t="s" s="2">
         <v>81</v>
@@ -7154,56 +7178,56 @@
         <v>81</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH45" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AI45" t="s" s="2">
-        <v>335</v>
+        <v>81</v>
       </c>
       <c r="AJ45" t="s" s="2">
         <v>102</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>81</v>
+        <v>329</v>
       </c>
       <c r="AL45" t="s" s="2">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="AM45" t="s" s="2">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="AN45" t="s" s="2">
-        <v>81</v>
+        <v>332</v>
       </c>
       <c r="AO45" t="s" s="2">
-        <v>327</v>
+        <v>333</v>
       </c>
     </row>
-    <row r="46" hidden="true">
+    <row r="46">
       <c r="A46" t="s" s="2">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
-        <v>81</v>
+        <v>335</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G46" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H46" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="I46" t="s" s="2">
         <v>81</v>
@@ -7212,18 +7236,18 @@
         <v>91</v>
       </c>
       <c r="K46" t="s" s="2">
+        <v>192</v>
+      </c>
+      <c r="L46" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="M46" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="N46" t="s" s="2">
         <v>338</v>
       </c>
-      <c r="L46" t="s" s="2">
-        <v>339</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="N46" s="2"/>
-      <c r="O46" t="s" s="2">
-        <v>341</v>
-      </c>
+      <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
         <v>81</v>
       </c>
@@ -7247,13 +7271,13 @@
         <v>81</v>
       </c>
       <c r="X46" t="s" s="2">
-        <v>81</v>
+        <v>298</v>
       </c>
       <c r="Y46" t="s" s="2">
-        <v>81</v>
+        <v>339</v>
       </c>
       <c r="Z46" t="s" s="2">
-        <v>81</v>
+        <v>340</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>81</v>
@@ -7271,16 +7295,16 @@
         <v>81</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH46" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AI46" t="s" s="2">
-        <v>81</v>
+        <v>341</v>
       </c>
       <c r="AJ46" t="s" s="2">
         <v>102</v>
@@ -7289,16 +7313,16 @@
         <v>81</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="AM46" t="s" s="2">
-        <v>342</v>
+        <v>331</v>
       </c>
       <c r="AN46" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AO46" t="s" s="2">
-        <v>81</v>
+        <v>333</v>
       </c>
     </row>
     <row r="47" hidden="true">
@@ -7314,7 +7338,7 @@
       </c>
       <c r="E47" s="2"/>
       <c r="F47" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="G47" t="s" s="2">
         <v>90</v>
@@ -7338,7 +7362,9 @@
         <v>346</v>
       </c>
       <c r="N47" s="2"/>
-      <c r="O47" s="2"/>
+      <c r="O47" t="s" s="2">
+        <v>347</v>
+      </c>
       <c r="P47" t="s" s="2">
         <v>81</v>
       </c>
@@ -7389,7 +7415,7 @@
         <v>343</v>
       </c>
       <c r="AG47" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="AH47" t="s" s="2">
         <v>90</v>
@@ -7401,35 +7427,35 @@
         <v>102</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>347</v>
+        <v>81</v>
       </c>
       <c r="AL47" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="AM47" t="s" s="2">
         <v>348</v>
       </c>
-      <c r="AM47" t="s" s="2">
-        <v>349</v>
-      </c>
       <c r="AN47" t="s" s="2">
-        <v>350</v>
+        <v>81</v>
       </c>
       <c r="AO47" t="s" s="2">
-        <v>351</v>
+        <v>81</v>
       </c>
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
-        <v>353</v>
+        <v>81</v>
       </c>
       <c r="E48" s="2"/>
       <c r="F48" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="G48" t="s" s="2">
         <v>90</v>
@@ -7444,13 +7470,13 @@
         <v>91</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -7501,10 +7527,10 @@
         <v>81</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="AG48" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="AH48" t="s" s="2">
         <v>90</v>
@@ -7516,41 +7542,41 @@
         <v>102</v>
       </c>
       <c r="AK48" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="AL48" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="AM48" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="AN48" t="s" s="2">
+        <v>356</v>
+      </c>
+      <c r="AO48" t="s" s="2">
         <v>357</v>
       </c>
-      <c r="AL48" t="s" s="2">
+    </row>
+    <row r="49" hidden="true">
+      <c r="A49" t="s" s="2">
         <v>358</v>
       </c>
-      <c r="AM48" t="s" s="2">
-        <v>359</v>
-      </c>
-      <c r="AN48" t="s" s="2">
-        <v>360</v>
-      </c>
-      <c r="AO48" t="s" s="2">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="s" s="2">
-        <v>362</v>
-      </c>
       <c r="B49" t="s" s="2">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="E49" s="2"/>
       <c r="F49" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="G49" t="s" s="2">
         <v>90</v>
       </c>
       <c r="H49" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="I49" t="s" s="2">
         <v>81</v>
@@ -7559,13 +7585,13 @@
         <v>91</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
@@ -7616,7 +7642,7 @@
         <v>81</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>79</v>
@@ -7631,41 +7657,41 @@
         <v>102</v>
       </c>
       <c r="AK49" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="AL49" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="AM49" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="AN49" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="AO49" t="s" s="2">
         <v>367</v>
       </c>
-      <c r="AL49" t="s" s="2">
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="2">
         <v>368</v>
       </c>
-      <c r="AM49" t="s" s="2">
-        <v>369</v>
-      </c>
-      <c r="AN49" t="s" s="2">
-        <v>370</v>
-      </c>
-      <c r="AO49" t="s" s="2">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="50" hidden="true">
-      <c r="A50" t="s" s="2">
-        <v>372</v>
-      </c>
       <c r="B50" t="s" s="2">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
-        <v>81</v>
+        <v>369</v>
       </c>
       <c r="E50" s="2"/>
       <c r="F50" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="G50" t="s" s="2">
         <v>90</v>
       </c>
       <c r="H50" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="I50" t="s" s="2">
         <v>81</v>
@@ -7674,13 +7700,13 @@
         <v>91</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -7707,13 +7733,13 @@
         <v>81</v>
       </c>
       <c r="X50" t="s" s="2">
-        <v>292</v>
+        <v>81</v>
       </c>
       <c r="Y50" t="s" s="2">
-        <v>376</v>
+        <v>81</v>
       </c>
       <c r="Z50" t="s" s="2">
-        <v>377</v>
+        <v>81</v>
       </c>
       <c r="AA50" t="s" s="2">
         <v>81</v>
@@ -7731,7 +7757,7 @@
         <v>81</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>79</v>
@@ -7746,31 +7772,31 @@
         <v>102</v>
       </c>
       <c r="AK50" t="s" s="2">
-        <v>81</v>
+        <v>373</v>
       </c>
       <c r="AL50" t="s" s="2">
-        <v>81</v>
+        <v>374</v>
       </c>
       <c r="AM50" t="s" s="2">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="AN50" t="s" s="2">
-        <v>81</v>
+        <v>376</v>
       </c>
       <c r="AO50" t="s" s="2">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
-        <v>381</v>
+        <v>81</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" t="s" s="2">
@@ -7789,13 +7815,13 @@
         <v>91</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
@@ -7822,13 +7848,13 @@
         <v>81</v>
       </c>
       <c r="X51" t="s" s="2">
-        <v>81</v>
+        <v>298</v>
       </c>
       <c r="Y51" t="s" s="2">
-        <v>81</v>
+        <v>382</v>
       </c>
       <c r="Z51" t="s" s="2">
-        <v>81</v>
+        <v>383</v>
       </c>
       <c r="AA51" t="s" s="2">
         <v>81</v>
@@ -7846,7 +7872,7 @@
         <v>81</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>79</v>
@@ -7861,31 +7887,31 @@
         <v>102</v>
       </c>
       <c r="AK51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM51" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="AN51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO51" t="s" s="2">
         <v>385</v>
       </c>
-      <c r="AL51" t="s" s="2">
+    </row>
+    <row r="52" hidden="true">
+      <c r="A52" t="s" s="2">
         <v>386</v>
       </c>
-      <c r="AM51" t="s" s="2">
-        <v>387</v>
-      </c>
-      <c r="AN51" t="s" s="2">
-        <v>388</v>
-      </c>
-      <c r="AO51" t="s" s="2">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="s" s="2">
-        <v>390</v>
-      </c>
       <c r="B52" t="s" s="2">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" t="s" s="2">
@@ -7895,7 +7921,7 @@
         <v>90</v>
       </c>
       <c r="H52" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="I52" t="s" s="2">
         <v>81</v>
@@ -7904,17 +7930,15 @@
         <v>91</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>394</v>
-      </c>
-      <c r="N52" t="s" s="2">
-        <v>395</v>
-      </c>
+        <v>390</v>
+      </c>
+      <c r="N52" s="2"/>
       <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
         <v>81</v>
@@ -7963,7 +7987,7 @@
         <v>81</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>79</v>
@@ -7978,31 +8002,31 @@
         <v>102</v>
       </c>
       <c r="AK52" t="s" s="2">
+        <v>391</v>
+      </c>
+      <c r="AL52" t="s" s="2">
+        <v>392</v>
+      </c>
+      <c r="AM52" t="s" s="2">
+        <v>393</v>
+      </c>
+      <c r="AN52" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="AO52" t="s" s="2">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="2">
         <v>396</v>
       </c>
-      <c r="AL52" t="s" s="2">
-        <v>397</v>
-      </c>
-      <c r="AM52" t="s" s="2">
-        <v>398</v>
-      </c>
-      <c r="AN52" t="s" s="2">
-        <v>399</v>
-      </c>
-      <c r="AO52" t="s" s="2">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="53" hidden="true">
-      <c r="A53" t="s" s="2">
-        <v>401</v>
-      </c>
       <c r="B53" t="s" s="2">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="E53" s="2"/>
       <c r="F53" t="s" s="2">
@@ -8012,7 +8036,7 @@
         <v>90</v>
       </c>
       <c r="H53" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="I53" t="s" s="2">
         <v>81</v>
@@ -8021,16 +8045,16 @@
         <v>91</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>192</v>
+        <v>398</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="N53" t="s" s="2">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="O53" s="2"/>
       <c r="P53" t="s" s="2">
@@ -8056,13 +8080,13 @@
         <v>81</v>
       </c>
       <c r="X53" t="s" s="2">
-        <v>292</v>
+        <v>81</v>
       </c>
       <c r="Y53" t="s" s="2">
-        <v>406</v>
+        <v>81</v>
       </c>
       <c r="Z53" t="s" s="2">
-        <v>407</v>
+        <v>81</v>
       </c>
       <c r="AA53" t="s" s="2">
         <v>81</v>
@@ -8080,7 +8104,7 @@
         <v>81</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>79</v>
@@ -8095,38 +8119,38 @@
         <v>102</v>
       </c>
       <c r="AK53" t="s" s="2">
-        <v>408</v>
+        <v>402</v>
       </c>
       <c r="AL53" t="s" s="2">
-        <v>409</v>
+        <v>403</v>
       </c>
       <c r="AM53" t="s" s="2">
-        <v>410</v>
+        <v>404</v>
       </c>
       <c r="AN53" t="s" s="2">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="AO53" t="s" s="2">
-        <v>81</v>
+        <v>406</v>
       </c>
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="E54" s="2"/>
       <c r="F54" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G54" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H54" t="s" s="2">
         <v>81</v>
@@ -8138,16 +8162,16 @@
         <v>91</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>414</v>
+        <v>192</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>415</v>
+        <v>409</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>416</v>
+        <v>410</v>
       </c>
       <c r="N54" t="s" s="2">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="O54" s="2"/>
       <c r="P54" t="s" s="2">
@@ -8173,13 +8197,13 @@
         <v>81</v>
       </c>
       <c r="X54" t="s" s="2">
-        <v>81</v>
+        <v>298</v>
       </c>
       <c r="Y54" t="s" s="2">
-        <v>81</v>
+        <v>412</v>
       </c>
       <c r="Z54" t="s" s="2">
-        <v>81</v>
+        <v>413</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>81</v>
@@ -8197,13 +8221,13 @@
         <v>81</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH54" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AI54" t="s" s="2">
         <v>81</v>
@@ -8212,16 +8236,16 @@
         <v>102</v>
       </c>
       <c r="AK54" t="s" s="2">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="AL54" t="s" s="2">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="AM54" t="s" s="2">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="AN54" t="s" s="2">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="AO54" t="s" s="2">
         <v>81</v>
@@ -8229,14 +8253,14 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
-        <v>81</v>
+        <v>419</v>
       </c>
       <c r="E55" s="2"/>
       <c r="F55" t="s" s="2">
@@ -8255,15 +8279,17 @@
         <v>91</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>192</v>
+        <v>420</v>
       </c>
       <c r="L55" t="s" s="2">
+        <v>421</v>
+      </c>
+      <c r="M55" t="s" s="2">
         <v>422</v>
       </c>
-      <c r="M55" t="s" s="2">
+      <c r="N55" t="s" s="2">
         <v>423</v>
       </c>
-      <c r="N55" s="2"/>
       <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
         <v>81</v>
@@ -8288,13 +8314,13 @@
         <v>81</v>
       </c>
       <c r="X55" t="s" s="2">
-        <v>292</v>
+        <v>81</v>
       </c>
       <c r="Y55" t="s" s="2">
-        <v>424</v>
+        <v>81</v>
       </c>
       <c r="Z55" t="s" s="2">
-        <v>425</v>
+        <v>81</v>
       </c>
       <c r="AA55" t="s" s="2">
         <v>81</v>
@@ -8312,7 +8338,7 @@
         <v>81</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>79</v>
@@ -8327,16 +8353,16 @@
         <v>102</v>
       </c>
       <c r="AK55" t="s" s="2">
-        <v>81</v>
+        <v>424</v>
       </c>
       <c r="AL55" t="s" s="2">
-        <v>81</v>
+        <v>425</v>
       </c>
       <c r="AM55" t="s" s="2">
         <v>426</v>
       </c>
       <c r="AN55" t="s" s="2">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="AO55" t="s" s="2">
         <v>81</v>
@@ -8370,10 +8396,10 @@
         <v>91</v>
       </c>
       <c r="K56" t="s" s="2">
+        <v>192</v>
+      </c>
+      <c r="L56" t="s" s="2">
         <v>428</v>
-      </c>
-      <c r="L56" t="s" s="2">
-        <v>422</v>
       </c>
       <c r="M56" t="s" s="2">
         <v>429</v>
@@ -8403,13 +8429,13 @@
         <v>81</v>
       </c>
       <c r="X56" t="s" s="2">
-        <v>81</v>
+        <v>298</v>
       </c>
       <c r="Y56" t="s" s="2">
-        <v>81</v>
+        <v>430</v>
       </c>
       <c r="Z56" t="s" s="2">
-        <v>81</v>
+        <v>431</v>
       </c>
       <c r="AA56" t="s" s="2">
         <v>81</v>
@@ -8448,10 +8474,10 @@
         <v>81</v>
       </c>
       <c r="AM56" t="s" s="2">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="AN56" t="s" s="2">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="AO56" t="s" s="2">
         <v>81</v>
@@ -8459,10 +8485,10 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8485,17 +8511,15 @@
         <v>91</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>192</v>
+        <v>434</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>433</v>
-      </c>
-      <c r="N57" t="s" s="2">
-        <v>434</v>
-      </c>
+        <v>435</v>
+      </c>
+      <c r="N57" s="2"/>
       <c r="O57" s="2"/>
       <c r="P57" t="s" s="2">
         <v>81</v>
@@ -8520,13 +8544,13 @@
         <v>81</v>
       </c>
       <c r="X57" t="s" s="2">
-        <v>292</v>
+        <v>81</v>
       </c>
       <c r="Y57" t="s" s="2">
-        <v>435</v>
+        <v>81</v>
       </c>
       <c r="Z57" t="s" s="2">
-        <v>436</v>
+        <v>81</v>
       </c>
       <c r="AA57" t="s" s="2">
         <v>81</v>
@@ -8544,7 +8568,7 @@
         <v>81</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>79</v>
@@ -8559,16 +8583,16 @@
         <v>102</v>
       </c>
       <c r="AK57" t="s" s="2">
-        <v>437</v>
+        <v>81</v>
       </c>
       <c r="AL57" t="s" s="2">
-        <v>438</v>
+        <v>81</v>
       </c>
       <c r="AM57" t="s" s="2">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="AN57" t="s" s="2">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="AO57" t="s" s="2">
         <v>81</v>
@@ -8576,10 +8600,10 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -8602,16 +8626,16 @@
         <v>91</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>442</v>
+        <v>192</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="N58" t="s" s="2">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
@@ -8637,13 +8661,13 @@
         <v>81</v>
       </c>
       <c r="X58" t="s" s="2">
-        <v>81</v>
+        <v>298</v>
       </c>
       <c r="Y58" t="s" s="2">
-        <v>81</v>
+        <v>441</v>
       </c>
       <c r="Z58" t="s" s="2">
-        <v>81</v>
+        <v>442</v>
       </c>
       <c r="AA58" t="s" s="2">
         <v>81</v>
@@ -8661,7 +8685,7 @@
         <v>81</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>79</v>
@@ -8676,16 +8700,16 @@
         <v>102</v>
       </c>
       <c r="AK58" t="s" s="2">
+        <v>443</v>
+      </c>
+      <c r="AL58" t="s" s="2">
+        <v>444</v>
+      </c>
+      <c r="AM58" t="s" s="2">
+        <v>445</v>
+      </c>
+      <c r="AN58" t="s" s="2">
         <v>446</v>
-      </c>
-      <c r="AL58" t="s" s="2">
-        <v>447</v>
-      </c>
-      <c r="AM58" t="s" s="2">
-        <v>448</v>
-      </c>
-      <c r="AN58" t="s" s="2">
-        <v>440</v>
       </c>
       <c r="AO58" t="s" s="2">
         <v>81</v>
@@ -8693,10 +8717,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -8716,18 +8740,20 @@
         <v>81</v>
       </c>
       <c r="J59" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="K59" t="s" s="2">
+        <v>448</v>
+      </c>
+      <c r="L59" t="s" s="2">
+        <v>449</v>
+      </c>
+      <c r="M59" t="s" s="2">
         <v>450</v>
       </c>
-      <c r="L59" t="s" s="2">
+      <c r="N59" t="s" s="2">
         <v>451</v>
       </c>
-      <c r="M59" t="s" s="2">
-        <v>452</v>
-      </c>
-      <c r="N59" s="2"/>
       <c r="O59" s="2"/>
       <c r="P59" t="s" s="2">
         <v>81</v>
@@ -8776,7 +8802,7 @@
         <v>81</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>79</v>
@@ -8791,16 +8817,16 @@
         <v>102</v>
       </c>
       <c r="AK59" t="s" s="2">
+        <v>452</v>
+      </c>
+      <c r="AL59" t="s" s="2">
         <v>453</v>
       </c>
-      <c r="AL59" t="s" s="2">
+      <c r="AM59" t="s" s="2">
         <v>454</v>
       </c>
-      <c r="AM59" t="s" s="2">
-        <v>455</v>
-      </c>
       <c r="AN59" t="s" s="2">
-        <v>81</v>
+        <v>446</v>
       </c>
       <c r="AO59" t="s" s="2">
         <v>81</v>
@@ -8808,14 +8834,14 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
-        <v>457</v>
+        <v>81</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" t="s" s="2">
@@ -8834,17 +8860,15 @@
         <v>81</v>
       </c>
       <c r="K60" t="s" s="2">
+        <v>456</v>
+      </c>
+      <c r="L60" t="s" s="2">
+        <v>457</v>
+      </c>
+      <c r="M60" t="s" s="2">
         <v>458</v>
       </c>
-      <c r="L60" t="s" s="2">
-        <v>459</v>
-      </c>
-      <c r="M60" t="s" s="2">
-        <v>460</v>
-      </c>
-      <c r="N60" t="s" s="2">
-        <v>461</v>
-      </c>
+      <c r="N60" s="2"/>
       <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
         <v>81</v>
@@ -8893,7 +8917,7 @@
         <v>81</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>79</v>
@@ -8908,13 +8932,13 @@
         <v>102</v>
       </c>
       <c r="AK60" t="s" s="2">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="AL60" t="s" s="2">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="AM60" t="s" s="2">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="AN60" t="s" s="2">
         <v>81</v>
@@ -8925,14 +8949,14 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
-        <v>81</v>
+        <v>463</v>
       </c>
       <c r="E61" s="2"/>
       <c r="F61" t="s" s="2">
@@ -8948,19 +8972,19 @@
         <v>81</v>
       </c>
       <c r="J61" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="K61" t="s" s="2">
+        <v>464</v>
+      </c>
+      <c r="L61" t="s" s="2">
+        <v>465</v>
+      </c>
+      <c r="M61" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="L61" t="s" s="2">
+      <c r="N61" t="s" s="2">
         <v>467</v>
-      </c>
-      <c r="M61" t="s" s="2">
-        <v>468</v>
-      </c>
-      <c r="N61" t="s" s="2">
-        <v>469</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
@@ -9010,7 +9034,7 @@
         <v>81</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>79</v>
@@ -9025,31 +9049,31 @@
         <v>102</v>
       </c>
       <c r="AK61" t="s" s="2">
-        <v>81</v>
+        <v>468</v>
       </c>
       <c r="AL61" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="AM61" t="s" s="2">
         <v>470</v>
       </c>
-      <c r="AM61" t="s" s="2">
+      <c r="AN61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO61" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="62" hidden="true">
+      <c r="A62" t="s" s="2">
         <v>471</v>
       </c>
-      <c r="AN61" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO61" t="s" s="2">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="s" s="2">
-        <v>472</v>
-      </c>
       <c r="B62" t="s" s="2">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
-        <v>473</v>
+        <v>81</v>
       </c>
       <c r="E62" s="2"/>
       <c r="F62" t="s" s="2">
@@ -9059,7 +9083,7 @@
         <v>80</v>
       </c>
       <c r="H62" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="I62" t="s" s="2">
         <v>81</v>
@@ -9068,20 +9092,18 @@
         <v>91</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>192</v>
+        <v>472</v>
       </c>
       <c r="L62" t="s" s="2">
+        <v>473</v>
+      </c>
+      <c r="M62" t="s" s="2">
         <v>474</v>
       </c>
-      <c r="M62" t="s" s="2">
+      <c r="N62" t="s" s="2">
         <v>475</v>
       </c>
-      <c r="N62" t="s" s="2">
-        <v>476</v>
-      </c>
-      <c r="O62" t="s" s="2">
-        <v>477</v>
-      </c>
+      <c r="O62" s="2"/>
       <c r="P62" t="s" s="2">
         <v>81</v>
       </c>
@@ -9105,11 +9127,13 @@
         <v>81</v>
       </c>
       <c r="X62" t="s" s="2">
-        <v>478</v>
-      </c>
-      <c r="Y62" s="2"/>
+        <v>81</v>
+      </c>
+      <c r="Y62" t="s" s="2">
+        <v>81</v>
+      </c>
       <c r="Z62" t="s" s="2">
-        <v>479</v>
+        <v>81</v>
       </c>
       <c r="AA62" t="s" s="2">
         <v>81</v>
@@ -9127,7 +9151,7 @@
         <v>81</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>79</v>
@@ -9145,28 +9169,28 @@
         <v>81</v>
       </c>
       <c r="AL62" t="s" s="2">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="AM62" t="s" s="2">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="AN62" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AO62" t="s" s="2">
-        <v>481</v>
+        <v>81</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
-        <v>81</v>
+        <v>479</v>
       </c>
       <c r="E63" s="2"/>
       <c r="F63" t="s" s="2">
@@ -9182,19 +9206,23 @@
         <v>81</v>
       </c>
       <c r="J63" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="K63" t="s" s="2">
+        <v>192</v>
+      </c>
+      <c r="L63" t="s" s="2">
+        <v>480</v>
+      </c>
+      <c r="M63" t="s" s="2">
+        <v>481</v>
+      </c>
+      <c r="N63" t="s" s="2">
+        <v>482</v>
+      </c>
+      <c r="O63" t="s" s="2">
         <v>483</v>
       </c>
-      <c r="L63" t="s" s="2">
-        <v>484</v>
-      </c>
-      <c r="M63" t="s" s="2">
-        <v>485</v>
-      </c>
-      <c r="N63" s="2"/>
-      <c r="O63" s="2"/>
       <c r="P63" t="s" s="2">
         <v>81</v>
       </c>
@@ -9218,13 +9246,11 @@
         <v>81</v>
       </c>
       <c r="X63" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Y63" t="s" s="2">
-        <v>81</v>
-      </c>
+        <v>484</v>
+      </c>
+      <c r="Y63" s="2"/>
       <c r="Z63" t="s" s="2">
-        <v>81</v>
+        <v>485</v>
       </c>
       <c r="AA63" t="s" s="2">
         <v>81</v>
@@ -9242,7 +9268,7 @@
         <v>81</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>79</v>
@@ -9257,27 +9283,27 @@
         <v>102</v>
       </c>
       <c r="AK63" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL63" t="s" s="2">
+        <v>476</v>
+      </c>
+      <c r="AM63" t="s" s="2">
         <v>486</v>
       </c>
-      <c r="AL63" t="s" s="2">
-        <v>336</v>
-      </c>
-      <c r="AM63" t="s" s="2">
+      <c r="AN63" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO63" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="AN63" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO63" t="s" s="2">
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="2">
         <v>488</v>
       </c>
-    </row>
-    <row r="64" hidden="true">
-      <c r="A64" t="s" s="2">
-        <v>489</v>
-      </c>
       <c r="B64" t="s" s="2">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9288,19 +9314,19 @@
         <v>79</v>
       </c>
       <c r="G64" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H64" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="I64" t="s" s="2">
         <v>81</v>
       </c>
       <c r="J64" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="K64" t="s" s="2">
-        <v>155</v>
+        <v>489</v>
       </c>
       <c r="L64" t="s" s="2">
         <v>490</v>
@@ -9357,13 +9383,13 @@
         <v>81</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH64" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AI64" t="s" s="2">
         <v>81</v>
@@ -9372,27 +9398,27 @@
         <v>102</v>
       </c>
       <c r="AK64" t="s" s="2">
-        <v>81</v>
+        <v>492</v>
       </c>
       <c r="AL64" t="s" s="2">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="AM64" t="s" s="2">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="AN64" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AO64" t="s" s="2">
-        <v>81</v>
+        <v>494</v>
       </c>
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -9403,7 +9429,7 @@
         <v>79</v>
       </c>
       <c r="G65" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H65" t="s" s="2">
         <v>81</v>
@@ -9412,20 +9438,18 @@
         <v>81</v>
       </c>
       <c r="J65" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="K65" t="s" s="2">
-        <v>494</v>
+        <v>155</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>496</v>
-      </c>
-      <c r="N65" t="s" s="2">
         <v>497</v>
       </c>
+      <c r="N65" s="2"/>
       <c r="O65" s="2"/>
       <c r="P65" t="s" s="2">
         <v>81</v>
@@ -9474,13 +9498,13 @@
         <v>81</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH65" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AI65" t="s" s="2">
         <v>81</v>
@@ -9489,23 +9513,140 @@
         <v>102</v>
       </c>
       <c r="AK65" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL65" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="AM65" t="s" s="2">
         <v>498</v>
       </c>
-      <c r="AL65" t="s" s="2">
+      <c r="AN65" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO65" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="66" hidden="true">
+      <c r="A66" t="s" s="2">
+        <v>499</v>
+      </c>
+      <c r="B66" t="s" s="2">
+        <v>499</v>
+      </c>
+      <c r="C66" s="2"/>
+      <c r="D66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E66" s="2"/>
+      <c r="F66" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G66" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="H66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="K66" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="L66" t="s" s="2">
+        <v>501</v>
+      </c>
+      <c r="M66" t="s" s="2">
+        <v>502</v>
+      </c>
+      <c r="N66" t="s" s="2">
+        <v>503</v>
+      </c>
+      <c r="O66" s="2"/>
+      <c r="P66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q66" s="2"/>
+      <c r="R66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF66" t="s" s="2">
+        <v>499</v>
+      </c>
+      <c r="AG66" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH66" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AI66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ66" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK66" t="s" s="2">
+        <v>504</v>
+      </c>
+      <c r="AL66" t="s" s="2">
         <v>133</v>
       </c>
-      <c r="AM65" t="s" s="2">
-        <v>499</v>
-      </c>
-      <c r="AN65" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO65" t="s" s="2">
+      <c r="AM66" t="s" s="2">
+        <v>505</v>
+      </c>
+      <c r="AN66" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO66" t="s" s="2">
         <v>81</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AO65">
+  <autoFilter ref="A1:AO66">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -9515,7 +9656,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI64">
+  <conditionalFormatting sqref="A2:AI65">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>